<commit_message>
fix(s1): only Субподрядчик and Заказчик in buyer files; test forbids third parties (#269 review)
Removes the Инвестор row from KS-2/KS-3 (cells unchanged) and the
«Иные участники» row from file 06, replaces the categorical sentence in
file 10 with the owner's wording, and widens the buyer-file check to
forbid Подрядчик, Генподрядчик, Инвестор and Иные участники as a class.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UmCUuQToGDpJHXok26LuA6
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/04-ks-2-ks-3.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/04-ks-2-ks-3.xlsx
@@ -512,14 +512,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Инвестор</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="n"/>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1544,11 +1536,10 @@
     </row>
     <row r="81"/>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="23">
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D6:H6"/>
-    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="D11:H11"/>
@@ -1565,7 +1556,6 @@
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="D15:H15"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D5:H5"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A80:H81"/>
@@ -1614,17 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Инвестор</t>
-        </is>
-      </c>
-      <c r="D5">
-        <f>'КС-2'!D5</f>
-        <v/>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1922,27 +1901,25 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="18">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A9:B9"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A8:B8"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="D6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>